<commit_message>
Add example gains/losses XLSX file
Sample eTrade export with 7 sell transactions (RS and ESPP)
using fake company symbol ACME, a summary row with correct
totals, and all 28 columns matching the real eTrade format.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/sample_gains_losses.xlsx
+++ b/examples/sample_gains_losses.xlsx
@@ -576,7 +576,7 @@
         <v>Sell</v>
       </c>
       <c r="B3" t="str">
-        <v>EBAY</v>
+        <v>ACME</v>
       </c>
       <c r="C3" t="str">
         <v>RS</v>
@@ -662,7 +662,7 @@
         <v>Sell</v>
       </c>
       <c r="B4" t="str">
-        <v>EBAY</v>
+        <v>ACME</v>
       </c>
       <c r="C4" t="str">
         <v>RS</v>
@@ -748,7 +748,7 @@
         <v>Sell</v>
       </c>
       <c r="B5" t="str">
-        <v>EBAY</v>
+        <v>ACME</v>
       </c>
       <c r="C5" t="str">
         <v>ESPP</v>
@@ -834,7 +834,7 @@
         <v>Sell</v>
       </c>
       <c r="B6" t="str">
-        <v>EBAY</v>
+        <v>ACME</v>
       </c>
       <c r="C6" t="str">
         <v>RS</v>
@@ -920,7 +920,7 @@
         <v>Sell</v>
       </c>
       <c r="B7" t="str">
-        <v>EBAY</v>
+        <v>ACME</v>
       </c>
       <c r="C7" t="str">
         <v>RS</v>
@@ -1006,7 +1006,7 @@
         <v>Sell</v>
       </c>
       <c r="B8" t="str">
-        <v>EBAY</v>
+        <v>ACME</v>
       </c>
       <c r="C8" t="str">
         <v>RS</v>
@@ -1092,7 +1092,7 @@
         <v>Sell</v>
       </c>
       <c r="B9" t="str">
-        <v>EBAY</v>
+        <v>ACME</v>
       </c>
       <c r="C9" t="str">
         <v>RS</v>

</xml_diff>